<commit_message>
Update SAAM Part 1/2 results, plots, and notebooks (carbon, TE, net-zero portfolios)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/resultsPart1/Template_for_Part_I_SAAM_FILLED.xlsx
+++ b/resultsPart1/Template_for_Part_I_SAAM_FILLED.xlsx
@@ -718,10 +718,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.07368513028127814</v>
+        <v>0.07368513028127816</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.07682359371139644</v>
+        <v>0.08297304640916292</v>
       </c>
       <c r="E3" s="22" t="n">
         <v>41640</v>
@@ -730,7 +730,7 @@
         <v>-0.04048947345151503</v>
       </c>
       <c r="G3" s="24" t="n">
-        <v>-0.03372043843105216</v>
+        <v>-0.02683435396305055</v>
       </c>
     </row>
     <row r="4">
@@ -743,7 +743,7 @@
         <v>0.1319812486575313</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.1082484001453696</v>
+        <v>0.1094799354129191</v>
       </c>
       <c r="E4" s="9" t="n">
         <v>41671</v>
@@ -752,7 +752,7 @@
         <v>0.02331943699437828</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.04371105140309498</v>
+        <v>0.03791328039808017</v>
       </c>
     </row>
     <row r="5">
@@ -765,7 +765,7 @@
         <v>0.06699265210726146</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.07338436159341799</v>
+        <v>0.07985198788651937</v>
       </c>
       <c r="E5" s="9" t="n">
         <v>41699</v>
@@ -774,7 +774,7 @@
         <v>0.003371766637113682</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0.008722043255537246</v>
+        <v>0.00520361391115977</v>
       </c>
     </row>
     <row r="6">
@@ -787,16 +787,16 @@
         <v>0.4268741817023679</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.5492495319487741</v>
+        <v>0.5974274559380806</v>
       </c>
       <c r="E6" s="9" t="n">
         <v>41730</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.008777486381004077</v>
+        <v>-0.008777486381004075</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.003321513760514499</v>
+        <v>-0.01248598836937543</v>
       </c>
     </row>
     <row r="7">
@@ -806,10 +806,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.1144225119748021</v>
+        <v>-0.114422511974802</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-0.09470271213460883</v>
+        <v>-0.08161278032634771</v>
       </c>
       <c r="E7" s="9" t="n">
         <v>41760</v>
@@ -818,7 +818,7 @@
         <v>0.03059397305135126</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>0.04051229218208836</v>
+        <v>0.05017855186410958</v>
       </c>
     </row>
     <row r="8">
@@ -831,16 +831,16 @@
         <v>0.1329161675884338</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.09892417251873023</v>
+        <v>0.1033084224012594</v>
       </c>
       <c r="E8" s="9" t="n">
         <v>41791</v>
       </c>
       <c r="F8" t="n">
-        <v>0.03366651966028278</v>
+        <v>0.03366651966028279</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.02745466963648263</v>
+        <v>0.04495775350079282</v>
       </c>
     </row>
     <row r="9">
@@ -866,7 +866,7 @@
         <v>0.01685100140992564</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0.01749485173877074</v>
+        <v>0.01479289503400832</v>
       </c>
     </row>
     <row r="10">
@@ -874,10 +874,10 @@
         <v>41852</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.009684462650971398</v>
+        <v>-0.0096844626509714</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0.01390158622497953</v>
+        <v>0.01316259125548763</v>
       </c>
     </row>
     <row r="11">
@@ -885,10 +885,10 @@
         <v>41883</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.03605195727030297</v>
+        <v>-0.03605195727030298</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>-0.02500074068114893</v>
+        <v>-0.02459569281239882</v>
       </c>
     </row>
     <row r="12">
@@ -897,10 +897,10 @@
         <v>41913</v>
       </c>
       <c r="F12" t="n">
-        <v>0.005930134348938088</v>
+        <v>0.005930134348938087</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0.04405298379114288</v>
+        <v>0.01716861196903664</v>
       </c>
     </row>
     <row r="13">
@@ -911,7 +911,7 @@
         <v>-0.009762737347359845</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>-0.006167541641332776</v>
+        <v>-0.002098241288190673</v>
       </c>
     </row>
     <row r="14">
@@ -922,7 +922,7 @@
         <v>-0.01219472194413195</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>-0.004510171715604626</v>
+        <v>-0.01104794834577141</v>
       </c>
     </row>
     <row r="15">
@@ -933,7 +933,7 @@
         <v>0.01586806528511714</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0.06435569974471414</v>
+        <v>0.06769796225234752</v>
       </c>
     </row>
     <row r="16">
@@ -941,10 +941,10 @@
         <v>42036</v>
       </c>
       <c r="F16" t="n">
-        <v>0.04942362362528413</v>
+        <v>0.04942362362528414</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0.007337447403532193</v>
+        <v>0.01005219245028276</v>
       </c>
     </row>
     <row r="17">
@@ -952,10 +952,10 @@
         <v>42064</v>
       </c>
       <c r="F17" t="n">
-        <v>0.001202914852920956</v>
+        <v>0.001202914852920955</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0.005274070800596021</v>
+        <v>0.009904205448856037</v>
       </c>
     </row>
     <row r="18">
@@ -966,7 +966,7 @@
         <v>0.03855697876271107</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0.008471784607219058</v>
+        <v>0.04844092319580841</v>
       </c>
     </row>
     <row r="19">
@@ -977,7 +977,7 @@
         <v>-0.001561251520133272</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>-0.01573433605483825</v>
+        <v>0.01417570670206102</v>
       </c>
     </row>
     <row r="20">
@@ -988,7 +988,7 @@
         <v>-0.02850356954529635</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>-0.02028820224241046</v>
+        <v>0.004639316465013753</v>
       </c>
     </row>
     <row r="21">
@@ -996,10 +996,10 @@
         <v>42186</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.00077053674696835</v>
+        <v>-0.0007705367469683509</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>0.04144108119613914</v>
+        <v>0.02513607953542246</v>
       </c>
     </row>
     <row r="22">
@@ -1010,7 +1010,7 @@
         <v>-0.08019499151490729</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>-0.04231808715954325</v>
+        <v>-0.05599795557293978</v>
       </c>
     </row>
     <row r="23">
@@ -1018,10 +1018,10 @@
         <v>42248</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.05461561032166429</v>
+        <v>-0.05461561032166427</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>0.006674658268978394</v>
+        <v>0.03569759440325317</v>
       </c>
     </row>
     <row r="24">
@@ -1032,7 +1032,7 @@
         <v>0.08948339042686859</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>0.05643893663944043</v>
+        <v>0.09957812539169746</v>
       </c>
     </row>
     <row r="25">
@@ -1040,10 +1040,10 @@
         <v>42309</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.00817924809061117</v>
+        <v>-0.008179248090611171</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>-0.03838253227367233</v>
+        <v>-0.04619220838289497</v>
       </c>
     </row>
     <row r="26">
@@ -1054,7 +1054,7 @@
         <v>0.01133223491474854</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>0.0360514937350866</v>
+        <v>0.07421998958734838</v>
       </c>
     </row>
     <row r="27">
@@ -1062,10 +1062,10 @@
         <v>42370</v>
       </c>
       <c r="F27" t="n">
-        <v>-0.08428095090786758</v>
+        <v>-0.08428095090786757</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>-0.03726052224751289</v>
+        <v>-0.04433351266147144</v>
       </c>
     </row>
     <row r="28">
@@ -1073,10 +1073,10 @@
         <v>42401</v>
       </c>
       <c r="F28" t="n">
-        <v>-0.02672314194639413</v>
+        <v>-0.02672314194639414</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0.008276399302456482</v>
+        <v>0.0147916721499332</v>
       </c>
     </row>
     <row r="29">
@@ -1087,7 +1087,7 @@
         <v>0.07415778085701943</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>0.05149799721916105</v>
+        <v>0.04869786627316838</v>
       </c>
     </row>
     <row r="30">
@@ -1095,10 +1095,10 @@
         <v>42461</v>
       </c>
       <c r="F30" t="n">
-        <v>0.03442984583439445</v>
+        <v>0.03442984583439446</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>0.001158474487485638</v>
+        <v>0.02682663580713714</v>
       </c>
     </row>
     <row r="31">
@@ -1109,7 +1109,7 @@
         <v>-0.01492715775055223</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>0.005232802384829737</v>
+        <v>-0.002193794381034996</v>
       </c>
     </row>
     <row r="32">
@@ -1120,7 +1120,7 @@
         <v>-0.01635436421676002</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0.01386476271981075</v>
+        <v>0.008193547018057554</v>
       </c>
     </row>
     <row r="33">
@@ -1131,7 +1131,7 @@
         <v>0.07153602239309542</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>0.04578616222663465</v>
+        <v>0.05419131802009266</v>
       </c>
     </row>
     <row r="34">
@@ -1139,10 +1139,10 @@
         <v>42583</v>
       </c>
       <c r="F34" t="n">
-        <v>1.205308435116921e-05</v>
+        <v>1.205308435116769e-05</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>-0.01484634216969547</v>
+        <v>-0.02804826564451434</v>
       </c>
     </row>
     <row r="35">
@@ -1153,7 +1153,7 @@
         <v>0.01763854255927381</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>0.02340321474553714</v>
+        <v>0.03386633552835684</v>
       </c>
     </row>
     <row r="36">
@@ -1161,10 +1161,10 @@
         <v>42644</v>
       </c>
       <c r="F36" t="n">
-        <v>0.008011040932537048</v>
+        <v>0.008011040932537046</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>-0.001786458211199128</v>
+        <v>-0.007419509607220094</v>
       </c>
     </row>
     <row r="37">
@@ -1172,10 +1172,10 @@
         <v>42675</v>
       </c>
       <c r="F37" t="n">
-        <v>-0.01705760290332942</v>
+        <v>-0.01705760290332941</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>-0.03243396544324695</v>
+        <v>-0.03826340350936401</v>
       </c>
     </row>
     <row r="38">
@@ -1183,10 +1183,10 @@
         <v>42705</v>
       </c>
       <c r="F38" t="n">
-        <v>0.006482280129466028</v>
+        <v>0.006482280129466026</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>-0.0222609863500437</v>
+        <v>-0.001954767674454246</v>
       </c>
     </row>
     <row r="39">
@@ -1197,7 +1197,7 @@
         <v>0.04135812637218023</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0.05311907974325426</v>
+        <v>0.04274727120314341</v>
       </c>
     </row>
     <row r="40">
@@ -1208,7 +1208,7 @@
         <v>0.02107198459456889</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>0.001283239181729237</v>
+        <v>0.007972044055475714</v>
       </c>
     </row>
     <row r="41">
@@ -1219,7 +1219,7 @@
         <v>0.007732858177485461</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>0.009655626711710144</v>
+        <v>0.01197541636034464</v>
       </c>
     </row>
     <row r="42">
@@ -1227,10 +1227,10 @@
         <v>42826</v>
       </c>
       <c r="F42" t="n">
-        <v>0.003585356840164128</v>
+        <v>0.003585356840164129</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0.006839238290687357</v>
+        <v>0.008466606323018303</v>
       </c>
     </row>
     <row r="43">
@@ -1241,7 +1241,7 @@
         <v>0.01454196468074921</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>0.05256686176964361</v>
+        <v>0.04635828395630238</v>
       </c>
     </row>
     <row r="44">
@@ -1249,10 +1249,10 @@
         <v>42887</v>
       </c>
       <c r="F44" t="n">
-        <v>0.01345422346375389</v>
+        <v>0.0134542234637539</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>-0.0005093726284566956</v>
+        <v>0.01099939832531105</v>
       </c>
     </row>
     <row r="45">
@@ -1260,10 +1260,10 @@
         <v>42917</v>
       </c>
       <c r="F45" t="n">
-        <v>0.03167035109072777</v>
+        <v>0.03167035109072776</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>0.02577997021946943</v>
+        <v>0.02322326835322486</v>
       </c>
     </row>
     <row r="46">
@@ -1271,10 +1271,10 @@
         <v>42948</v>
       </c>
       <c r="F46" t="n">
-        <v>0.0002686130151001249</v>
+        <v>0.0002686130151001229</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>0.001328297230861215</v>
+        <v>-7.824680119127795e-05</v>
       </c>
     </row>
     <row r="47">
@@ -1282,10 +1282,10 @@
         <v>42979</v>
       </c>
       <c r="F47" t="n">
-        <v>0.009240972539303897</v>
+        <v>0.009240972539303895</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>-0.01637222049578039</v>
+        <v>-0.007920305406882768</v>
       </c>
     </row>
     <row r="48">
@@ -1293,10 +1293,10 @@
         <v>43009</v>
       </c>
       <c r="F48" t="n">
-        <v>0.03387370024092356</v>
+        <v>0.03387370024092355</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0.02196767459777964</v>
+        <v>0.02666135298185091</v>
       </c>
     </row>
     <row r="49">
@@ -1307,7 +1307,7 @@
         <v>0.02225376187045875</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>0.02942330074908188</v>
+        <v>0.0302797307164832</v>
       </c>
     </row>
     <row r="50">
@@ -1318,7 +1318,7 @@
         <v>0.01618716016572429</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>-0.02146365688679248</v>
+        <v>0.003947377201369198</v>
       </c>
     </row>
     <row r="51">
@@ -1326,10 +1326,10 @@
         <v>43101</v>
       </c>
       <c r="F51" t="n">
-        <v>0.04389335150817856</v>
+        <v>0.04389335150817857</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>0.02542354347796055</v>
+        <v>0.03468211384772182</v>
       </c>
     </row>
     <row r="52">
@@ -1337,10 +1337,10 @@
         <v>43132</v>
       </c>
       <c r="F52" t="n">
-        <v>-0.02527834884320104</v>
+        <v>-0.02527834884320103</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>-0.009672059531116755</v>
+        <v>-0.0182783402968558</v>
       </c>
     </row>
     <row r="53">
@@ -1348,10 +1348,10 @@
         <v>43160</v>
       </c>
       <c r="F53" t="n">
-        <v>-0.02830604716912869</v>
+        <v>-0.0283060471691287</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0.005945906345682046</v>
+        <v>-0.004419129878341129</v>
       </c>
     </row>
     <row r="54">
@@ -1362,7 +1362,7 @@
         <v>0.01340684869621066</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.006471057708557043</v>
+        <v>0.003060869570273047</v>
       </c>
     </row>
     <row r="55">
@@ -1370,10 +1370,10 @@
         <v>43221</v>
       </c>
       <c r="F55" t="n">
-        <v>-0.008639777072155116</v>
+        <v>-0.008639777072155115</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>-0.00674862011082352</v>
+        <v>-0.006140311204996303</v>
       </c>
     </row>
     <row r="56">
@@ -1384,7 +1384,7 @@
         <v>-0.01711392942793056</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>-0.01171471974123706</v>
+        <v>-0.01704381690759118</v>
       </c>
     </row>
     <row r="57">
@@ -1395,7 +1395,7 @@
         <v>0.01394725132902852</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>0.006164668178423137</v>
+        <v>-0.005192429068399358</v>
       </c>
     </row>
     <row r="58">
@@ -1406,7 +1406,7 @@
         <v>-0.009841112947684229</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>-0.004004205425535015</v>
+        <v>-0.01390004580516111</v>
       </c>
     </row>
     <row r="59">
@@ -1414,10 +1414,10 @@
         <v>43344</v>
       </c>
       <c r="F59" t="n">
-        <v>0.01747505828020535</v>
+        <v>0.01747505828020536</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0.02194850802566573</v>
+        <v>0.01953507101524213</v>
       </c>
     </row>
     <row r="60">
@@ -1425,10 +1425,10 @@
         <v>43374</v>
       </c>
       <c r="F60" t="n">
-        <v>-0.07987975005622826</v>
+        <v>-0.07987975005622824</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>-0.05273794264054638</v>
+        <v>-0.06298352008287902</v>
       </c>
     </row>
     <row r="61">
@@ -1439,7 +1439,7 @@
         <v>0.01044717997512502</v>
       </c>
       <c r="G61" s="2" t="n">
-        <v>-0.004069997945490143</v>
+        <v>0.01341475506797758</v>
       </c>
     </row>
     <row r="62">
@@ -1450,7 +1450,7 @@
         <v>-0.0474872847379031</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>-0.01309820199685491</v>
+        <v>-0.02556821344196983</v>
       </c>
     </row>
     <row r="63">
@@ -1458,10 +1458,10 @@
         <v>43466</v>
       </c>
       <c r="F63" t="n">
-        <v>0.06297387877447772</v>
+        <v>0.0629738787744777</v>
       </c>
       <c r="G63" s="2" t="n">
-        <v>0.03441301903649543</v>
+        <v>0.04748528215187577</v>
       </c>
     </row>
     <row r="64">
@@ -1472,7 +1472,7 @@
         <v>0.01307141981360736</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>0.0008412160274516759</v>
+        <v>-0.002496812836022413</v>
       </c>
     </row>
     <row r="65">
@@ -1480,10 +1480,10 @@
         <v>43525</v>
       </c>
       <c r="F65" t="n">
-        <v>0.008996699289400651</v>
+        <v>0.008996699289400655</v>
       </c>
       <c r="G65" s="2" t="n">
-        <v>-0.01571663064324622</v>
+        <v>-0.005733510492336729</v>
       </c>
     </row>
     <row r="66">
@@ -1494,7 +1494,7 @@
         <v>0.01438508065744196</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>-0.02466318308360773</v>
+        <v>-0.01748378516335002</v>
       </c>
     </row>
     <row r="67">
@@ -1502,10 +1502,10 @@
         <v>43586</v>
       </c>
       <c r="F67" t="n">
-        <v>-0.03766184416881432</v>
+        <v>-0.0376618441688143</v>
       </c>
       <c r="G67" s="2" t="n">
-        <v>-0.008358243083743196</v>
+        <v>-0.02281170717001003</v>
       </c>
     </row>
     <row r="68">
@@ -1513,10 +1513,10 @@
         <v>43617</v>
       </c>
       <c r="F68" t="n">
-        <v>0.04465900754985221</v>
+        <v>0.0446590075498522</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>0.006174581612178536</v>
+        <v>0.02917123987838828</v>
       </c>
     </row>
     <row r="69">
@@ -1524,10 +1524,10 @@
         <v>43647</v>
       </c>
       <c r="F69" t="n">
-        <v>-0.001478025915951289</v>
+        <v>-0.001478025915951288</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>-0.01087120355778368</v>
+        <v>-0.003033594892416819</v>
       </c>
     </row>
     <row r="70">
@@ -1535,10 +1535,10 @@
         <v>43678</v>
       </c>
       <c r="F70" t="n">
-        <v>-0.02953219588787843</v>
+        <v>-0.02953219588787844</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>-0.02331179294509975</v>
+        <v>-0.02081380002765265</v>
       </c>
     </row>
     <row r="71">
@@ -1546,10 +1546,10 @@
         <v>43709</v>
       </c>
       <c r="F71" t="n">
-        <v>0.03169675369381878</v>
+        <v>0.03169675369381877</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>0.03199976708403471</v>
+        <v>0.02416243928157943</v>
       </c>
     </row>
     <row r="72">
@@ -1557,10 +1557,10 @@
         <v>43739</v>
       </c>
       <c r="F72" t="n">
-        <v>0.04222503010332254</v>
+        <v>0.04222503010332255</v>
       </c>
       <c r="G72" s="2" t="n">
-        <v>0.02373930970828995</v>
+        <v>0.03465975489045085</v>
       </c>
     </row>
     <row r="73">
@@ -1568,10 +1568,10 @@
         <v>43770</v>
       </c>
       <c r="F73" t="n">
-        <v>0.0006623396556880351</v>
+        <v>0.0006623396556880356</v>
       </c>
       <c r="G73" s="2" t="n">
-        <v>-0.008942097806136666</v>
+        <v>-0.001375951204651958</v>
       </c>
     </row>
     <row r="74">
@@ -1579,10 +1579,10 @@
         <v>43800</v>
       </c>
       <c r="F74" t="n">
-        <v>0.02658707330149481</v>
+        <v>0.02658707330149482</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>0.02935934941609491</v>
+        <v>0.02007069367729969</v>
       </c>
     </row>
     <row r="75">
@@ -1593,7 +1593,7 @@
         <v>-0.01814376999091697</v>
       </c>
       <c r="G75" s="2" t="n">
-        <v>-0.01347531763241185</v>
+        <v>-0.01773419323667593</v>
       </c>
     </row>
     <row r="76">
@@ -1601,10 +1601,10 @@
         <v>43862</v>
       </c>
       <c r="F76" t="n">
-        <v>-0.08249361081516098</v>
+        <v>-0.08249361081516095</v>
       </c>
       <c r="G76" s="2" t="n">
-        <v>-0.05446430595235988</v>
+        <v>-0.08161278032634771</v>
       </c>
     </row>
     <row r="77">
@@ -1612,10 +1612,10 @@
         <v>43891</v>
       </c>
       <c r="F77" t="n">
-        <v>-0.1144225119748021</v>
+        <v>-0.114422511974802</v>
       </c>
       <c r="G77" s="2" t="n">
-        <v>-0.05967444433302653</v>
+        <v>-0.06749450506763345</v>
       </c>
     </row>
     <row r="78">
@@ -1623,10 +1623,10 @@
         <v>43922</v>
       </c>
       <c r="F78" t="n">
-        <v>0.06571679089092804</v>
+        <v>0.06571679089092802</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>0.0572740630714293</v>
+        <v>0.02622535933193653</v>
       </c>
     </row>
     <row r="79">
@@ -1634,10 +1634,10 @@
         <v>43952</v>
       </c>
       <c r="F79" t="n">
-        <v>0.03326311885969748</v>
+        <v>0.03326311885969749</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>-0.009605561437627464</v>
+        <v>0.00603156862737747</v>
       </c>
     </row>
     <row r="80">
@@ -1648,7 +1648,7 @@
         <v>0.02212671541778877</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>-0.008478502925631327</v>
+        <v>-0.003988777653338119</v>
       </c>
     </row>
     <row r="81">
@@ -1656,10 +1656,10 @@
         <v>44013</v>
       </c>
       <c r="F81" t="n">
-        <v>-0.007133950791691717</v>
+        <v>-0.007133950791691721</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>-0.02595095633485131</v>
+        <v>-0.01534364597033293</v>
       </c>
     </row>
     <row r="82">
@@ -1667,10 +1667,10 @@
         <v>44044</v>
       </c>
       <c r="F82" t="n">
-        <v>0.06659854055011022</v>
+        <v>0.06659854055011025</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>0.05167116982420898</v>
+        <v>0.0547940566017449</v>
       </c>
     </row>
     <row r="83">
@@ -1681,7 +1681,7 @@
         <v>-0.01558211816931885</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>-0.02172825886019409</v>
+        <v>-0.02247113890148191</v>
       </c>
     </row>
     <row r="84">
@@ -1692,7 +1692,7 @@
         <v>-0.01114711037749189</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>-0.02865126062815581</v>
+        <v>-0.03332149400994699</v>
       </c>
     </row>
     <row r="85">
@@ -1703,7 +1703,7 @@
         <v>0.1329161675884338</v>
       </c>
       <c r="G85" s="2" t="n">
-        <v>0.0495357684620552</v>
+        <v>0.0846972596511165</v>
       </c>
     </row>
     <row r="86">
@@ -1714,7 +1714,7 @@
         <v>0.04500289559550905</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>0.01419979983304067</v>
+        <v>0.03396947745609171</v>
       </c>
     </row>
     <row r="87">
@@ -1722,10 +1722,10 @@
         <v>44197</v>
       </c>
       <c r="F87" t="n">
-        <v>-0.004358344985541992</v>
+        <v>-0.004358344985541991</v>
       </c>
       <c r="G87" s="2" t="n">
-        <v>0.02034058187724064</v>
+        <v>0.01630710652102</v>
       </c>
     </row>
     <row r="88">
@@ -1736,7 +1736,7 @@
         <v>0.02972893323740994</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>-0.004081841617305553</v>
+        <v>-0.004608768891539114</v>
       </c>
     </row>
     <row r="89">
@@ -1747,7 +1747,7 @@
         <v>0.01490585554540916</v>
       </c>
       <c r="G89" s="2" t="n">
-        <v>0.03396013313645612</v>
+        <v>0.0317153084340998</v>
       </c>
     </row>
     <row r="90">
@@ -1758,7 +1758,7 @@
         <v>-0.002097564848618794</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>-0.01386291701383349</v>
+        <v>-0.002737705221392509</v>
       </c>
     </row>
     <row r="91">
@@ -1766,10 +1766,10 @@
         <v>44317</v>
       </c>
       <c r="F91" t="n">
-        <v>0.02177273193545508</v>
+        <v>0.02177273193545509</v>
       </c>
       <c r="G91" s="2" t="n">
-        <v>0.01307574309669999</v>
+        <v>0.01143442704993856</v>
       </c>
     </row>
     <row r="92">
@@ -1777,10 +1777,10 @@
         <v>44348</v>
       </c>
       <c r="F92" t="n">
-        <v>-0.009546970987800166</v>
+        <v>-0.009546970987800172</v>
       </c>
       <c r="G92" s="2" t="n">
-        <v>0.001254153809581109</v>
+        <v>0.0001055065876696078</v>
       </c>
     </row>
     <row r="93">
@@ -1788,10 +1788,10 @@
         <v>44378</v>
       </c>
       <c r="F93" t="n">
-        <v>-0.01865403357871891</v>
+        <v>-0.01865403357871892</v>
       </c>
       <c r="G93" s="2" t="n">
-        <v>0.0157393178365074</v>
+        <v>-0.008911525350164876</v>
       </c>
     </row>
     <row r="94">
@@ -1802,7 +1802,7 @@
         <v>0.02351596473738751</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>0.02235054638099317</v>
+        <v>0.02733412707403294</v>
       </c>
     </row>
     <row r="95">
@@ -1810,10 +1810,10 @@
         <v>44440</v>
       </c>
       <c r="F95" t="n">
-        <v>0.01202228137420931</v>
+        <v>0.01202228137420932</v>
       </c>
       <c r="G95" s="2" t="n">
-        <v>0.009295143718100108</v>
+        <v>0.009589284977846562</v>
       </c>
     </row>
     <row r="96">
@@ -1824,7 +1824,7 @@
         <v>-0.01192907893722273</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>-0.01375789703703588</v>
+        <v>-0.01598223160520491</v>
       </c>
     </row>
     <row r="97">
@@ -1835,7 +1835,7 @@
         <v>-0.03824791607430596</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>-0.009972394916567085</v>
+        <v>-0.02760678033825098</v>
       </c>
     </row>
     <row r="98">
@@ -1843,10 +1843,10 @@
         <v>44531</v>
       </c>
       <c r="F98" t="n">
-        <v>0.02944009693036797</v>
+        <v>0.02944009693036796</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>0.01902353911501541</v>
+        <v>0.01556425240429478</v>
       </c>
     </row>
     <row r="99">
@@ -1854,10 +1854,10 @@
         <v>44562</v>
       </c>
       <c r="F99" t="n">
-        <v>-0.03375044271505787</v>
+        <v>-0.03375044271505785</v>
       </c>
       <c r="G99" s="2" t="n">
-        <v>-0.003182032361377544</v>
+        <v>-0.01413895394175397</v>
       </c>
     </row>
     <row r="100">
@@ -1865,10 +1865,10 @@
         <v>44593</v>
       </c>
       <c r="F100" t="n">
-        <v>0.002150097697197571</v>
+        <v>0.002150097697197572</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>0.01606145942550081</v>
+        <v>0.01331697790362408</v>
       </c>
     </row>
     <row r="101">
@@ -1879,7 +1879,7 @@
         <v>0.01664911367265891</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>-0.02710329777317858</v>
+        <v>-0.02062269915927131</v>
       </c>
     </row>
     <row r="102">
@@ -1890,7 +1890,7 @@
         <v>-0.06831217236867652</v>
       </c>
       <c r="G102" s="2" t="n">
-        <v>-0.02646288867024614</v>
+        <v>-0.03653211832684621</v>
       </c>
     </row>
     <row r="103">
@@ -1898,10 +1898,10 @@
         <v>44682</v>
       </c>
       <c r="F103" t="n">
-        <v>0.008690514569214441</v>
+        <v>0.008690514569214445</v>
       </c>
       <c r="G103" s="2" t="n">
-        <v>0.02282164210116965</v>
+        <v>0.01570605645146273</v>
       </c>
     </row>
     <row r="104">
@@ -1909,10 +1909,10 @@
         <v>44713</v>
       </c>
       <c r="F104" t="n">
-        <v>-0.0713748681738695</v>
+        <v>-0.07137486817386951</v>
       </c>
       <c r="G104" s="2" t="n">
-        <v>-0.0682846721760417</v>
+        <v>-0.0409215650664142</v>
       </c>
     </row>
     <row r="105">
@@ -1920,10 +1920,10 @@
         <v>44743</v>
       </c>
       <c r="F105" t="n">
-        <v>0.04215114084727579</v>
+        <v>0.04215114084727578</v>
       </c>
       <c r="G105" s="2" t="n">
-        <v>0.02940424392881943</v>
+        <v>0.02662232085578096</v>
       </c>
     </row>
     <row r="106">
@@ -1934,7 +1934,7 @@
         <v>-0.02062739908050899</v>
       </c>
       <c r="G106" s="2" t="n">
-        <v>-0.02413592099026787</v>
+        <v>-0.01573585020258284</v>
       </c>
     </row>
     <row r="107">
@@ -1945,7 +1945,7 @@
         <v>-0.1006463825719439</v>
       </c>
       <c r="G107" s="2" t="n">
-        <v>-0.06485415318494556</v>
+        <v>-0.07126442838689748</v>
       </c>
     </row>
     <row r="108">
@@ -1953,10 +1953,10 @@
         <v>44835</v>
       </c>
       <c r="F108" t="n">
-        <v>0.01365951208600224</v>
+        <v>0.01365951208600223</v>
       </c>
       <c r="G108" s="2" t="n">
-        <v>-0.02673579272252086</v>
+        <v>-0.02370497349991343</v>
       </c>
     </row>
     <row r="109">
@@ -1967,7 +1967,7 @@
         <v>0.1089904939655742</v>
       </c>
       <c r="G109" s="2" t="n">
-        <v>0.09325845390090623</v>
+        <v>0.1033084224012594</v>
       </c>
     </row>
     <row r="110">
@@ -1978,7 +1978,7 @@
         <v>0.001797707029514407</v>
       </c>
       <c r="G110" s="2" t="n">
-        <v>0.02608679851263993</v>
+        <v>-0.008270467427200775</v>
       </c>
     </row>
     <row r="111">
@@ -1986,10 +1986,10 @@
         <v>44927</v>
       </c>
       <c r="F111" t="n">
-        <v>0.06470321798872862</v>
+        <v>0.06470321798872859</v>
       </c>
       <c r="G111" s="2" t="n">
-        <v>0.03635769933895575</v>
+        <v>0.03575590480213588</v>
       </c>
     </row>
     <row r="112">
@@ -2000,7 +2000,7 @@
         <v>-0.04510569340905411</v>
       </c>
       <c r="G112" s="2" t="n">
-        <v>-0.04194365304543823</v>
+        <v>-0.03731852460760221</v>
       </c>
     </row>
     <row r="113">
@@ -2008,10 +2008,10 @@
         <v>44986</v>
       </c>
       <c r="F113" t="n">
-        <v>0.02698098379847663</v>
+        <v>0.02698098379847662</v>
       </c>
       <c r="G113" s="2" t="n">
-        <v>0.04610412260103747</v>
+        <v>0.03506806033475651</v>
       </c>
     </row>
     <row r="114">
@@ -2019,10 +2019,10 @@
         <v>45017</v>
       </c>
       <c r="F114" t="n">
-        <v>0.006926623632841846</v>
+        <v>0.006926623632841845</v>
       </c>
       <c r="G114" s="2" t="n">
-        <v>0.03620010569350403</v>
+        <v>0.02363475003853821</v>
       </c>
     </row>
     <row r="115">
@@ -2030,10 +2030,10 @@
         <v>45047</v>
       </c>
       <c r="F115" t="n">
-        <v>-0.00896759097369045</v>
+        <v>-0.008967590973690452</v>
       </c>
       <c r="G115" s="2" t="n">
-        <v>-0.01181653097251066</v>
+        <v>-0.008271366943441895</v>
       </c>
     </row>
     <row r="116">
@@ -2044,7 +2044,7 @@
         <v>0.04594594762545304</v>
       </c>
       <c r="G116" s="2" t="n">
-        <v>0.03087450653582883</v>
+        <v>0.02284520165073884</v>
       </c>
     </row>
     <row r="117">
@@ -2052,10 +2052,10 @@
         <v>45108</v>
       </c>
       <c r="F117" t="n">
-        <v>0.03775404095517168</v>
+        <v>0.03775404095517169</v>
       </c>
       <c r="G117" s="2" t="n">
-        <v>0.03395158216328445</v>
+        <v>0.02904423267542939</v>
       </c>
     </row>
     <row r="118">
@@ -2063,10 +2063,10 @@
         <v>45139</v>
       </c>
       <c r="F118" t="n">
-        <v>-0.03151863659945758</v>
+        <v>-0.03151863659945757</v>
       </c>
       <c r="G118" s="2" t="n">
-        <v>0.008257639268869105</v>
+        <v>-0.0080735049503928</v>
       </c>
     </row>
     <row r="119">
@@ -2077,7 +2077,7 @@
         <v>-0.0172917743383237</v>
       </c>
       <c r="G119" s="2" t="n">
-        <v>-0.006326741259521643</v>
+        <v>-0.01597027054338626</v>
       </c>
     </row>
     <row r="120">
@@ -2085,10 +2085,10 @@
         <v>45200</v>
       </c>
       <c r="F120" t="n">
-        <v>-0.05045691850664138</v>
+        <v>-0.05045691850664139</v>
       </c>
       <c r="G120" s="2" t="n">
-        <v>-0.01759585935855468</v>
+        <v>-0.02345860679142632</v>
       </c>
     </row>
     <row r="121">
@@ -2096,10 +2096,10 @@
         <v>45231</v>
       </c>
       <c r="F121" t="n">
-        <v>0.06964735184969617</v>
+        <v>0.06964735184969614</v>
       </c>
       <c r="G121" s="2" t="n">
-        <v>-0.09470271213460883</v>
+        <v>-0.00499835983894412</v>
       </c>
     </row>
     <row r="122">
@@ -2107,10 +2107,10 @@
         <v>45261</v>
       </c>
       <c r="F122" t="n">
-        <v>0.0516480067382371</v>
+        <v>0.05164800673823711</v>
       </c>
       <c r="G122" s="2" t="n">
-        <v>0.06360078272008131</v>
+        <v>0.0567587192559616</v>
       </c>
     </row>
     <row r="123">
@@ -2121,7 +2121,7 @@
         <v>0.02182857618970565</v>
       </c>
       <c r="G123" s="2" t="n">
-        <v>0.01268295036048629</v>
+        <v>0.0111518059730275</v>
       </c>
     </row>
     <row r="124">
@@ -2132,7 +2132,7 @@
         <v>0.02723204524390988</v>
       </c>
       <c r="G124" s="2" t="n">
-        <v>0.004019961571042908</v>
+        <v>-0.00173655103975348</v>
       </c>
     </row>
     <row r="125">
@@ -2143,7 +2143,7 @@
         <v>0.02524587861875428</v>
       </c>
       <c r="G125" s="2" t="n">
-        <v>0.04343717749510304</v>
+        <v>0.02805259883784097</v>
       </c>
     </row>
     <row r="126">
@@ -2154,7 +2154,7 @@
         <v>-0.03475389758867845</v>
       </c>
       <c r="G126" s="2" t="n">
-        <v>-0.03517275585620618</v>
+        <v>-0.02410646856753424</v>
       </c>
     </row>
     <row r="127">
@@ -2162,10 +2162,10 @@
         <v>45413</v>
       </c>
       <c r="F127" t="n">
-        <v>0.01196510662235035</v>
+        <v>0.01196510662235034</v>
       </c>
       <c r="G127" s="2" t="n">
-        <v>-0.009961454046910911</v>
+        <v>-0.01423044483292312</v>
       </c>
     </row>
     <row r="128">
@@ -2173,10 +2173,10 @@
         <v>45444</v>
       </c>
       <c r="F128" t="n">
-        <v>-0.005777866332475413</v>
+        <v>-0.005777866332475412</v>
       </c>
       <c r="G128" s="2" t="n">
-        <v>-0.02350407954929813</v>
+        <v>-0.0241460718255382</v>
       </c>
     </row>
     <row r="129">
@@ -2187,7 +2187,7 @@
         <v>0.04816725487792622</v>
       </c>
       <c r="G129" s="2" t="n">
-        <v>0.04571914926969616</v>
+        <v>0.04899698786181501</v>
       </c>
     </row>
     <row r="130">
@@ -2195,10 +2195,10 @@
         <v>45505</v>
       </c>
       <c r="F130" t="n">
-        <v>0.01417762556353757</v>
+        <v>0.01417762556353758</v>
       </c>
       <c r="G130" s="2" t="n">
-        <v>0.02468097832553223</v>
+        <v>0.01712719537325144</v>
       </c>
     </row>
     <row r="131">
@@ -2209,7 +2209,7 @@
         <v>0.02043168751973485</v>
       </c>
       <c r="G131" s="2" t="n">
-        <v>0.002513667665495675</v>
+        <v>0.01441072319064343</v>
       </c>
     </row>
     <row r="132">
@@ -2220,7 +2220,7 @@
         <v>-0.04388213536566083</v>
       </c>
       <c r="G132" s="2" t="n">
-        <v>-0.04028489138430813</v>
+        <v>-0.04314579080071766</v>
       </c>
     </row>
     <row r="133">
@@ -2228,10 +2228,10 @@
         <v>45597</v>
       </c>
       <c r="F133" t="n">
-        <v>0.003179359263831081</v>
+        <v>0.003179359263831083</v>
       </c>
       <c r="G133" s="2" t="n">
-        <v>0.02635128628065522</v>
+        <v>0.01880611660121303</v>
       </c>
     </row>
     <row r="134">
@@ -2239,10 +2239,10 @@
         <v>45627</v>
       </c>
       <c r="F134" t="n">
-        <v>-0.009904936314324882</v>
+        <v>-0.009904936314324887</v>
       </c>
       <c r="G134" s="2" t="n">
-        <v>-0.01882596565656548</v>
+        <v>-0.01380257567843542</v>
       </c>
     </row>
     <row r="135">
@@ -2250,10 +2250,10 @@
         <v>45658</v>
       </c>
       <c r="F135" t="n">
-        <v>0.0147328108169443</v>
+        <v>0.01473281081694431</v>
       </c>
       <c r="G135" s="2" t="n">
-        <v>0.04771157286152089</v>
+        <v>0.01042421168796662</v>
       </c>
     </row>
     <row r="136">
@@ -2261,10 +2261,10 @@
         <v>45689</v>
       </c>
       <c r="F136" t="n">
-        <v>-0.008825849403990399</v>
+        <v>-0.008825849403990397</v>
       </c>
       <c r="G136" s="2" t="n">
-        <v>0.04550113419923661</v>
+        <v>0.01310553285336153</v>
       </c>
     </row>
     <row r="137">
@@ -2272,10 +2272,10 @@
         <v>45717</v>
       </c>
       <c r="F137" t="n">
-        <v>0.004034043447141261</v>
+        <v>0.004034043447141258</v>
       </c>
       <c r="G137" s="2" t="n">
-        <v>0.04175227601296243</v>
+        <v>0.02877367932037785</v>
       </c>
     </row>
     <row r="138">
@@ -2283,10 +2283,10 @@
         <v>45748</v>
       </c>
       <c r="F138" t="n">
-        <v>0.05506506557113955</v>
+        <v>0.05506506557113954</v>
       </c>
       <c r="G138" s="2" t="n">
-        <v>0.09892417251873023</v>
+        <v>0.06032597440740353</v>
       </c>
     </row>
     <row r="139">
@@ -2297,7 +2297,7 @@
         <v>0.03866117694017075</v>
       </c>
       <c r="G139" s="2" t="n">
-        <v>0.01103062224175287</v>
+        <v>0.02099747500810106</v>
       </c>
     </row>
     <row r="140">
@@ -2308,7 +2308,7 @@
         <v>0.02285892640434826</v>
       </c>
       <c r="G140" s="2" t="n">
-        <v>0.04674701650791976</v>
+        <v>0.02969433149487082</v>
       </c>
     </row>
     <row r="141">
@@ -2316,10 +2316,10 @@
         <v>45839</v>
       </c>
       <c r="F141" t="n">
-        <v>-0.0002265904128584483</v>
+        <v>-0.0002265904128584473</v>
       </c>
       <c r="G141" s="2" t="n">
-        <v>0.0173144513928091</v>
+        <v>0.01592855190449243</v>
       </c>
     </row>
     <row r="142">
@@ -2327,10 +2327,10 @@
         <v>45870</v>
       </c>
       <c r="F142" t="n">
-        <v>0.06166295025496488</v>
+        <v>0.0616629502549649</v>
       </c>
       <c r="G142" s="2" t="n">
-        <v>0.01520982667870195</v>
+        <v>0.06241016406866283</v>
       </c>
     </row>
     <row r="143">
@@ -2341,7 +2341,7 @@
         <v>0.02037228912621098</v>
       </c>
       <c r="G143" s="2" t="n">
-        <v>0.02317667896131992</v>
+        <v>0.01155991273318836</v>
       </c>
     </row>
     <row r="144">
@@ -2352,7 +2352,7 @@
         <v>0.02807268951678298</v>
       </c>
       <c r="G144" s="2" t="n">
-        <v>-0.01314824841272121</v>
+        <v>-0.005064219238300935</v>
       </c>
     </row>
     <row r="145">
@@ -2360,10 +2360,10 @@
         <v>45962</v>
       </c>
       <c r="F145" t="n">
-        <v>-0.006469133677908644</v>
+        <v>-0.006469133677908642</v>
       </c>
       <c r="G145" s="2" t="n">
-        <v>0.02688327352050644</v>
+        <v>0.02685021106538299</v>
       </c>
     </row>
     <row r="146">
@@ -2371,10 +2371,10 @@
         <v>45992</v>
       </c>
       <c r="F146" s="4" t="n">
-        <v>0.007292430941722381</v>
+        <v>0.007292430941722384</v>
       </c>
       <c r="G146" s="5" t="n">
-        <v>0.0133575211198519</v>
+        <v>-0.007060512442369751</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Commit 13/05 at 5PM
</commit_message>
<xml_diff>
--- a/resultsPart1/Template_for_Part_I_SAAM_FILLED.xlsx
+++ b/resultsPart1/Template_for_Part_I_SAAM_FILLED.xlsx
@@ -718,19 +718,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.07368513028127816</v>
+        <v>0.07368513028127814</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.08297304640916292</v>
+        <v>0.07682647198193558</v>
       </c>
       <c r="E3" s="22" t="n">
         <v>41640</v>
       </c>
       <c r="F3" s="23" t="n">
-        <v>-0.04048947345151503</v>
+        <v>-0.04048947345151504</v>
       </c>
       <c r="G3" s="24" t="n">
-        <v>-0.02683435396305055</v>
+        <v>-0.03372043887629989</v>
       </c>
     </row>
     <row r="4">
@@ -743,7 +743,7 @@
         <v>0.1319812486575313</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.1094799354129191</v>
+        <v>0.1082492756956537</v>
       </c>
       <c r="E4" s="9" t="n">
         <v>41671</v>
@@ -752,7 +752,7 @@
         <v>0.02331943699437828</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.03791328039808017</v>
+        <v>0.04371105349788166</v>
       </c>
     </row>
     <row r="5">
@@ -762,19 +762,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.06699265210726146</v>
+        <v>0.06699265210726124</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.07985198788651937</v>
+        <v>0.07338733400997066</v>
       </c>
       <c r="E5" s="9" t="n">
         <v>41699</v>
       </c>
       <c r="F5" t="n">
-        <v>0.003371766637113682</v>
+        <v>0.003371766637113683</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0.00520361391115977</v>
+        <v>0.008722042209679563</v>
       </c>
     </row>
     <row r="6">
@@ -784,19 +784,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.4268741817023679</v>
+        <v>0.4268741817023678</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.5974274559380806</v>
+        <v>0.5492715119970986</v>
       </c>
       <c r="E6" s="9" t="n">
         <v>41730</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.008777486381004075</v>
+        <v>-0.008777486381004073</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>-0.01248598836937543</v>
+        <v>0.003321514019910478</v>
       </c>
     </row>
     <row r="7">
@@ -806,10 +806,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.114422511974802</v>
+        <v>-0.1144225119748021</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-0.08161278032634771</v>
+        <v>-0.09470271811091882</v>
       </c>
       <c r="E7" s="9" t="n">
         <v>41760</v>
@@ -818,7 +818,7 @@
         <v>0.03059397305135126</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>0.05017855186410958</v>
+        <v>0.04051229223988735</v>
       </c>
     </row>
     <row r="8">
@@ -831,16 +831,16 @@
         <v>0.1329161675884338</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.1033084224012594</v>
+        <v>0.09892414747185098</v>
       </c>
       <c r="E8" s="9" t="n">
         <v>41791</v>
       </c>
       <c r="F8" t="n">
-        <v>0.03366651966028279</v>
+        <v>0.03366651966028278</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0.04495775350079282</v>
+        <v>0.02745466930943692</v>
       </c>
     </row>
     <row r="9">
@@ -866,7 +866,7 @@
         <v>0.01685100140992564</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0.01479289503400832</v>
+        <v>0.01749485092991888</v>
       </c>
     </row>
     <row r="10">
@@ -874,10 +874,10 @@
         <v>41852</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.0096844626509714</v>
+        <v>-0.009684462650971396</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0.01316259125548763</v>
+        <v>0.0139015890134859</v>
       </c>
     </row>
     <row r="11">
@@ -885,10 +885,10 @@
         <v>41883</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.03605195727030298</v>
+        <v>-0.03605195727030297</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>-0.02459569281239882</v>
+        <v>-0.02500073963336744</v>
       </c>
     </row>
     <row r="12">
@@ -897,10 +897,10 @@
         <v>41913</v>
       </c>
       <c r="F12" t="n">
-        <v>0.005930134348938087</v>
+        <v>0.005930134348938085</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0.01716861196903664</v>
+        <v>0.04405298567858871</v>
       </c>
     </row>
     <row r="13">
@@ -908,10 +908,10 @@
         <v>41944</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.009762737347359845</v>
+        <v>-0.009762737347359843</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>-0.002098241288190673</v>
+        <v>-0.006167544413070214</v>
       </c>
     </row>
     <row r="14">
@@ -922,7 +922,7 @@
         <v>-0.01219472194413195</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>-0.01104794834577141</v>
+        <v>-0.004510172764650271</v>
       </c>
     </row>
     <row r="15">
@@ -933,7 +933,7 @@
         <v>0.01586806528511714</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0.06769796225234752</v>
+        <v>0.06435627519675433</v>
       </c>
     </row>
     <row r="16">
@@ -944,7 +944,7 @@
         <v>0.04942362362528414</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0.01005219245028276</v>
+        <v>0.007323482218085248</v>
       </c>
     </row>
     <row r="17">
@@ -952,10 +952,10 @@
         <v>42064</v>
       </c>
       <c r="F17" t="n">
-        <v>0.001202914852920955</v>
+        <v>0.001202914852920954</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0.009904205448856037</v>
+        <v>0.005272821589139426</v>
       </c>
     </row>
     <row r="18">
@@ -963,10 +963,10 @@
         <v>42095</v>
       </c>
       <c r="F18" t="n">
-        <v>0.03855697876271107</v>
+        <v>0.03855697876271106</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0.04844092319580841</v>
+        <v>0.008470393107070364</v>
       </c>
     </row>
     <row r="19">
@@ -974,10 +974,10 @@
         <v>42125</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.001561251520133272</v>
+        <v>-0.001561251520133274</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>0.01417570670206102</v>
+        <v>-0.01573443882362594</v>
       </c>
     </row>
     <row r="20">
@@ -988,7 +988,7 @@
         <v>-0.02850356954529635</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>0.004639316465013753</v>
+        <v>-0.02026010024919428</v>
       </c>
     </row>
     <row r="21">
@@ -996,10 +996,10 @@
         <v>42186</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.0007705367469683509</v>
+        <v>-0.0007705367469683513</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>0.02513607953542246</v>
+        <v>0.04147051694647307</v>
       </c>
     </row>
     <row r="22">
@@ -1010,7 +1010,7 @@
         <v>-0.08019499151490729</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>-0.05599795557293978</v>
+        <v>-0.04232159312270032</v>
       </c>
     </row>
     <row r="23">
@@ -1021,7 +1021,7 @@
         <v>-0.05461561032166427</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>0.03569759440325317</v>
+        <v>0.006677016125679486</v>
       </c>
     </row>
     <row r="24">
@@ -1032,7 +1032,7 @@
         <v>0.08948339042686859</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>0.09957812539169746</v>
+        <v>0.05643739020900651</v>
       </c>
     </row>
     <row r="25">
@@ -1040,10 +1040,10 @@
         <v>42309</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.008179248090611171</v>
+        <v>-0.008179248090611168</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>-0.04619220838289497</v>
+        <v>-0.03839389260432888</v>
       </c>
     </row>
     <row r="26">
@@ -1051,10 +1051,10 @@
         <v>42339</v>
       </c>
       <c r="F26" t="n">
-        <v>0.01133223491474854</v>
+        <v>0.01133223491474855</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>0.07421998958734838</v>
+        <v>0.03605899139397949</v>
       </c>
     </row>
     <row r="27">
@@ -1065,7 +1065,7 @@
         <v>-0.08428095090786757</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>-0.04433351266147144</v>
+        <v>-0.03726052029160455</v>
       </c>
     </row>
     <row r="28">
@@ -1076,7 +1076,7 @@
         <v>-0.02672314194639414</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0.0147916721499332</v>
+        <v>0.008276408746584866</v>
       </c>
     </row>
     <row r="29">
@@ -1087,7 +1087,7 @@
         <v>0.07415778085701943</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>0.04869786627316838</v>
+        <v>0.0514979778429837</v>
       </c>
     </row>
     <row r="30">
@@ -1095,10 +1095,10 @@
         <v>42461</v>
       </c>
       <c r="F30" t="n">
-        <v>0.03442984583439446</v>
+        <v>0.03442984583439445</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>0.02682663580713714</v>
+        <v>0.001158474800465909</v>
       </c>
     </row>
     <row r="31">
@@ -1109,7 +1109,7 @@
         <v>-0.01492715775055223</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>-0.002193794381034996</v>
+        <v>0.005232795190610201</v>
       </c>
     </row>
     <row r="32">
@@ -1120,7 +1120,7 @@
         <v>-0.01635436421676002</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0.008193547018057554</v>
+        <v>0.0138647766228471</v>
       </c>
     </row>
     <row r="33">
@@ -1131,7 +1131,7 @@
         <v>0.07153602239309542</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>0.05419131802009266</v>
+        <v>0.04578615765407262</v>
       </c>
     </row>
     <row r="34">
@@ -1139,10 +1139,10 @@
         <v>42583</v>
       </c>
       <c r="F34" t="n">
-        <v>1.205308435116769e-05</v>
+        <v>1.205308435116704e-05</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>-0.02804826564451434</v>
+        <v>-0.0148463583954585</v>
       </c>
     </row>
     <row r="35">
@@ -1153,7 +1153,7 @@
         <v>0.01763854255927381</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>0.03386633552835684</v>
+        <v>0.02340322287579565</v>
       </c>
     </row>
     <row r="36">
@@ -1161,10 +1161,10 @@
         <v>42644</v>
       </c>
       <c r="F36" t="n">
-        <v>0.008011040932537046</v>
+        <v>0.008011040932537048</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>-0.007419509607220094</v>
+        <v>-0.001786466809149536</v>
       </c>
     </row>
     <row r="37">
@@ -1172,10 +1172,10 @@
         <v>42675</v>
       </c>
       <c r="F37" t="n">
-        <v>-0.01705760290332941</v>
+        <v>-0.01705760290332942</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>-0.03826340350936401</v>
+        <v>-0.03243396959994697</v>
       </c>
     </row>
     <row r="38">
@@ -1186,7 +1186,7 @@
         <v>0.006482280129466026</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>-0.001954767674454246</v>
+        <v>-0.02226098739287418</v>
       </c>
     </row>
     <row r="39">
@@ -1197,7 +1197,7 @@
         <v>0.04135812637218023</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0.04274727120314341</v>
+        <v>0.05311908292266625</v>
       </c>
     </row>
     <row r="40">
@@ -1208,7 +1208,7 @@
         <v>0.02107198459456889</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>0.007972044055475714</v>
+        <v>0.001283233532351241</v>
       </c>
     </row>
     <row r="41">
@@ -1216,10 +1216,10 @@
         <v>42795</v>
       </c>
       <c r="F41" t="n">
-        <v>0.007732858177485461</v>
+        <v>0.007732858177485458</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>0.01197541636034464</v>
+        <v>0.009655624899508225</v>
       </c>
     </row>
     <row r="42">
@@ -1227,10 +1227,10 @@
         <v>42826</v>
       </c>
       <c r="F42" t="n">
-        <v>0.003585356840164129</v>
+        <v>0.00358535684016413</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0.008466606323018303</v>
+        <v>0.006839241226299838</v>
       </c>
     </row>
     <row r="43">
@@ -1238,10 +1238,10 @@
         <v>42856</v>
       </c>
       <c r="F43" t="n">
-        <v>0.01454196468074921</v>
+        <v>0.01454196468074922</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>0.04635828395630238</v>
+        <v>0.05256685961136696</v>
       </c>
     </row>
     <row r="44">
@@ -1249,10 +1249,10 @@
         <v>42887</v>
       </c>
       <c r="F44" t="n">
-        <v>0.0134542234637539</v>
+        <v>0.01345422346375389</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0.01099939832531105</v>
+        <v>-0.0005093710520899312</v>
       </c>
     </row>
     <row r="45">
@@ -1263,7 +1263,7 @@
         <v>0.03167035109072776</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>0.02322326835322486</v>
+        <v>0.0257799721253339</v>
       </c>
     </row>
     <row r="46">
@@ -1271,10 +1271,10 @@
         <v>42948</v>
       </c>
       <c r="F46" t="n">
-        <v>0.0002686130151001229</v>
+        <v>0.0002686130151001245</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>-7.824680119127795e-05</v>
+        <v>0.001328299441665514</v>
       </c>
     </row>
     <row r="47">
@@ -1282,10 +1282,10 @@
         <v>42979</v>
       </c>
       <c r="F47" t="n">
-        <v>0.009240972539303895</v>
+        <v>0.009240972539303897</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>-0.007920305406882768</v>
+        <v>-0.01637221734149759</v>
       </c>
     </row>
     <row r="48">
@@ -1293,10 +1293,10 @@
         <v>43009</v>
       </c>
       <c r="F48" t="n">
-        <v>0.03387370024092355</v>
+        <v>0.03387370024092354</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0.02666135298185091</v>
+        <v>0.0219676748988812</v>
       </c>
     </row>
     <row r="49">
@@ -1307,7 +1307,7 @@
         <v>0.02225376187045875</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>0.0302797307164832</v>
+        <v>0.02942329980506144</v>
       </c>
     </row>
     <row r="50">
@@ -1315,10 +1315,10 @@
         <v>43070</v>
       </c>
       <c r="F50" t="n">
-        <v>0.01618716016572429</v>
+        <v>0.01618716016572428</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>0.003947377201369198</v>
+        <v>-0.0214636525537239</v>
       </c>
     </row>
     <row r="51">
@@ -1329,7 +1329,7 @@
         <v>0.04389335150817857</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>0.03468211384772182</v>
+        <v>0.02542353970607091</v>
       </c>
     </row>
     <row r="52">
@@ -1340,7 +1340,7 @@
         <v>-0.02527834884320103</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>-0.0182783402968558</v>
+        <v>-0.009672067874833852</v>
       </c>
     </row>
     <row r="53">
@@ -1351,7 +1351,7 @@
         <v>-0.0283060471691287</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>-0.004419129878341129</v>
+        <v>0.005945896826180138</v>
       </c>
     </row>
     <row r="54">
@@ -1362,7 +1362,7 @@
         <v>0.01340684869621066</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.003060869570273047</v>
+        <v>0.006471059183300714</v>
       </c>
     </row>
     <row r="55">
@@ -1373,7 +1373,7 @@
         <v>-0.008639777072155115</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>-0.006140311204996303</v>
+        <v>-0.006748613850102703</v>
       </c>
     </row>
     <row r="56">
@@ -1384,7 +1384,7 @@
         <v>-0.01711392942793056</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>-0.01704381690759118</v>
+        <v>-0.01171471053301321</v>
       </c>
     </row>
     <row r="57">
@@ -1395,7 +1395,7 @@
         <v>0.01394725132902852</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>-0.005192429068399358</v>
+        <v>0.006164676200188038</v>
       </c>
     </row>
     <row r="58">
@@ -1403,10 +1403,10 @@
         <v>43313</v>
       </c>
       <c r="F58" t="n">
-        <v>-0.009841112947684229</v>
+        <v>-0.009841112947684231</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>-0.01390004580516111</v>
+        <v>-0.0040041885525491</v>
       </c>
     </row>
     <row r="59">
@@ -1417,7 +1417,7 @@
         <v>0.01747505828020536</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0.01953507101524213</v>
+        <v>0.0219485127410413</v>
       </c>
     </row>
     <row r="60">
@@ -1425,10 +1425,10 @@
         <v>43374</v>
       </c>
       <c r="F60" t="n">
-        <v>-0.07987975005622824</v>
+        <v>-0.07987975005622826</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>-0.06298352008287902</v>
+        <v>-0.05273795210175686</v>
       </c>
     </row>
     <row r="61">
@@ -1439,7 +1439,7 @@
         <v>0.01044717997512502</v>
       </c>
       <c r="G61" s="2" t="n">
-        <v>0.01341475506797758</v>
+        <v>-0.004070006621912522</v>
       </c>
     </row>
     <row r="62">
@@ -1450,7 +1450,7 @@
         <v>-0.0474872847379031</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>-0.02556821344196983</v>
+        <v>-0.01309820114761365</v>
       </c>
     </row>
     <row r="63">
@@ -1458,10 +1458,10 @@
         <v>43466</v>
       </c>
       <c r="F63" t="n">
-        <v>0.0629738787744777</v>
+        <v>0.06297387877447773</v>
       </c>
       <c r="G63" s="2" t="n">
-        <v>0.04748528215187577</v>
+        <v>0.03441301860459286</v>
       </c>
     </row>
     <row r="64">
@@ -1469,10 +1469,10 @@
         <v>43497</v>
       </c>
       <c r="F64" t="n">
-        <v>0.01307141981360736</v>
+        <v>0.01307141981360735</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>-0.002496812836022413</v>
+        <v>0.000841209138392239</v>
       </c>
     </row>
     <row r="65">
@@ -1480,10 +1480,10 @@
         <v>43525</v>
       </c>
       <c r="F65" t="n">
-        <v>0.008996699289400655</v>
+        <v>0.008996699289400651</v>
       </c>
       <c r="G65" s="2" t="n">
-        <v>-0.005733510492336729</v>
+        <v>-0.01571662787874445</v>
       </c>
     </row>
     <row r="66">
@@ -1494,7 +1494,7 @@
         <v>0.01438508065744196</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>-0.01748378516335002</v>
+        <v>-0.02466318172269521</v>
       </c>
     </row>
     <row r="67">
@@ -1502,10 +1502,10 @@
         <v>43586</v>
       </c>
       <c r="F67" t="n">
-        <v>-0.0376618441688143</v>
+        <v>-0.03766184416881434</v>
       </c>
       <c r="G67" s="2" t="n">
-        <v>-0.02281170717001003</v>
+        <v>-0.008358244411239052</v>
       </c>
     </row>
     <row r="68">
@@ -1513,10 +1513,10 @@
         <v>43617</v>
       </c>
       <c r="F68" t="n">
-        <v>0.0446590075498522</v>
+        <v>0.04465900754985221</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>0.02917123987838828</v>
+        <v>0.006174584951159891</v>
       </c>
     </row>
     <row r="69">
@@ -1524,10 +1524,10 @@
         <v>43647</v>
       </c>
       <c r="F69" t="n">
-        <v>-0.001478025915951288</v>
+        <v>-0.001478025915951289</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>-0.003033594892416819</v>
+        <v>-0.01087120557686846</v>
       </c>
     </row>
     <row r="70">
@@ -1538,7 +1538,7 @@
         <v>-0.02953219588787844</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>-0.02081380002765265</v>
+        <v>-0.02331179673818006</v>
       </c>
     </row>
     <row r="71">
@@ -1546,10 +1546,10 @@
         <v>43709</v>
       </c>
       <c r="F71" t="n">
-        <v>0.03169675369381877</v>
+        <v>0.03169675369381879</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>0.02416243928157943</v>
+        <v>0.03199976845295838</v>
       </c>
     </row>
     <row r="72">
@@ -1557,10 +1557,10 @@
         <v>43739</v>
       </c>
       <c r="F72" t="n">
-        <v>0.04222503010332255</v>
+        <v>0.04222503010332256</v>
       </c>
       <c r="G72" s="2" t="n">
-        <v>0.03465975489045085</v>
+        <v>0.02373931373878203</v>
       </c>
     </row>
     <row r="73">
@@ -1568,10 +1568,10 @@
         <v>43770</v>
       </c>
       <c r="F73" t="n">
-        <v>0.0006623396556880356</v>
+        <v>0.0006623396556880361</v>
       </c>
       <c r="G73" s="2" t="n">
-        <v>-0.001375951204651958</v>
+        <v>-0.008942091623270192</v>
       </c>
     </row>
     <row r="74">
@@ -1582,7 +1582,7 @@
         <v>0.02658707330149482</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>0.02007069367729969</v>
+        <v>0.0293593516425477</v>
       </c>
     </row>
     <row r="75">
@@ -1593,7 +1593,7 @@
         <v>-0.01814376999091697</v>
       </c>
       <c r="G75" s="2" t="n">
-        <v>-0.01773419323667593</v>
+        <v>-0.01347532322368908</v>
       </c>
     </row>
     <row r="76">
@@ -1601,10 +1601,10 @@
         <v>43862</v>
       </c>
       <c r="F76" t="n">
-        <v>-0.08249361081516095</v>
+        <v>-0.08249361081516096</v>
       </c>
       <c r="G76" s="2" t="n">
-        <v>-0.08161278032634771</v>
+        <v>-0.05446430737531551</v>
       </c>
     </row>
     <row r="77">
@@ -1612,10 +1612,10 @@
         <v>43891</v>
       </c>
       <c r="F77" t="n">
-        <v>-0.114422511974802</v>
+        <v>-0.1144225119748021</v>
       </c>
       <c r="G77" s="2" t="n">
-        <v>-0.06749450506763345</v>
+        <v>-0.05967442235619473</v>
       </c>
     </row>
     <row r="78">
@@ -1623,10 +1623,10 @@
         <v>43922</v>
       </c>
       <c r="F78" t="n">
-        <v>0.06571679089092802</v>
+        <v>0.06571679089092804</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>0.02622535933193653</v>
+        <v>0.05727404646993401</v>
       </c>
     </row>
     <row r="79">
@@ -1634,10 +1634,10 @@
         <v>43952</v>
       </c>
       <c r="F79" t="n">
-        <v>0.03326311885969749</v>
+        <v>0.03326311885969748</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>0.00603156862737747</v>
+        <v>-0.009605558719234755</v>
       </c>
     </row>
     <row r="80">
@@ -1648,7 +1648,7 @@
         <v>0.02212671541778877</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>-0.003988777653338119</v>
+        <v>-0.008478502024611043</v>
       </c>
     </row>
     <row r="81">
@@ -1659,7 +1659,7 @@
         <v>-0.007133950791691721</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>-0.01534364597033293</v>
+        <v>-0.02595095030205055</v>
       </c>
     </row>
     <row r="82">
@@ -1667,10 +1667,10 @@
         <v>44044</v>
       </c>
       <c r="F82" t="n">
-        <v>0.06659854055011025</v>
+        <v>0.06659854055011023</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>0.0547940566017449</v>
+        <v>0.05167117104153762</v>
       </c>
     </row>
     <row r="83">
@@ -1681,7 +1681,7 @@
         <v>-0.01558211816931885</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>-0.02247113890148191</v>
+        <v>-0.02172825228026486</v>
       </c>
     </row>
     <row r="84">
@@ -1689,10 +1689,10 @@
         <v>44105</v>
       </c>
       <c r="F84" t="n">
-        <v>-0.01114711037749189</v>
+        <v>-0.01114711037749188</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>-0.03332149400994699</v>
+        <v>-0.02865126012768907</v>
       </c>
     </row>
     <row r="85">
@@ -1703,7 +1703,7 @@
         <v>0.1329161675884338</v>
       </c>
       <c r="G85" s="2" t="n">
-        <v>0.0846972596511165</v>
+        <v>0.04953576687905507</v>
       </c>
     </row>
     <row r="86">
@@ -1714,7 +1714,7 @@
         <v>0.04500289559550905</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>0.03396947745609171</v>
+        <v>0.01419980390740913</v>
       </c>
     </row>
     <row r="87">
@@ -1722,10 +1722,10 @@
         <v>44197</v>
       </c>
       <c r="F87" t="n">
-        <v>-0.004358344985541991</v>
+        <v>-0.004358344985541989</v>
       </c>
       <c r="G87" s="2" t="n">
-        <v>0.01630710652102</v>
+        <v>0.02034058157277327</v>
       </c>
     </row>
     <row r="88">
@@ -1733,10 +1733,10 @@
         <v>44228</v>
       </c>
       <c r="F88" t="n">
-        <v>0.02972893323740994</v>
+        <v>0.02972893323740993</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>-0.004608768891539114</v>
+        <v>-0.004081841298610376</v>
       </c>
     </row>
     <row r="89">
@@ -1744,10 +1744,10 @@
         <v>44256</v>
       </c>
       <c r="F89" t="n">
-        <v>0.01490585554540916</v>
+        <v>0.01490585554540915</v>
       </c>
       <c r="G89" s="2" t="n">
-        <v>0.0317153084340998</v>
+        <v>0.03396013314218618</v>
       </c>
     </row>
     <row r="90">
@@ -1758,7 +1758,7 @@
         <v>-0.002097564848618794</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>-0.002737705221392509</v>
+        <v>-0.01386291617550004</v>
       </c>
     </row>
     <row r="91">
@@ -1766,10 +1766,10 @@
         <v>44317</v>
       </c>
       <c r="F91" t="n">
-        <v>0.02177273193545509</v>
+        <v>0.0217727319354551</v>
       </c>
       <c r="G91" s="2" t="n">
-        <v>0.01143442704993856</v>
+        <v>0.01307574349255962</v>
       </c>
     </row>
     <row r="92">
@@ -1777,10 +1777,10 @@
         <v>44348</v>
       </c>
       <c r="F92" t="n">
-        <v>-0.009546970987800172</v>
+        <v>-0.009546970987800168</v>
       </c>
       <c r="G92" s="2" t="n">
-        <v>0.0001055065876696078</v>
+        <v>0.001254154286012045</v>
       </c>
     </row>
     <row r="93">
@@ -1788,10 +1788,10 @@
         <v>44378</v>
       </c>
       <c r="F93" t="n">
-        <v>-0.01865403357871892</v>
+        <v>-0.01865403357871891</v>
       </c>
       <c r="G93" s="2" t="n">
-        <v>-0.008911525350164876</v>
+        <v>0.01573931734718008</v>
       </c>
     </row>
     <row r="94">
@@ -1802,7 +1802,7 @@
         <v>0.02351596473738751</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>0.02733412707403294</v>
+        <v>0.02235054664931814</v>
       </c>
     </row>
     <row r="95">
@@ -1813,7 +1813,7 @@
         <v>0.01202228137420932</v>
       </c>
       <c r="G95" s="2" t="n">
-        <v>0.009589284977846562</v>
+        <v>0.009295143586449351</v>
       </c>
     </row>
     <row r="96">
@@ -1824,7 +1824,7 @@
         <v>-0.01192907893722273</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>-0.01598223160520491</v>
+        <v>-0.01375789717015077</v>
       </c>
     </row>
     <row r="97">
@@ -1835,7 +1835,7 @@
         <v>-0.03824791607430596</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>-0.02760678033825098</v>
+        <v>-0.009972394579582112</v>
       </c>
     </row>
     <row r="98">
@@ -1846,7 +1846,7 @@
         <v>0.02944009693036796</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>0.01556425240429478</v>
+        <v>0.01902353912009314</v>
       </c>
     </row>
     <row r="99">
@@ -1854,10 +1854,10 @@
         <v>44562</v>
       </c>
       <c r="F99" t="n">
-        <v>-0.03375044271505785</v>
+        <v>-0.03375044271505787</v>
       </c>
       <c r="G99" s="2" t="n">
-        <v>-0.01413895394175397</v>
+        <v>-0.003182029855407728</v>
       </c>
     </row>
     <row r="100">
@@ -1865,10 +1865,10 @@
         <v>44593</v>
       </c>
       <c r="F100" t="n">
-        <v>0.002150097697197572</v>
+        <v>0.002150097697197569</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>0.01331697790362408</v>
+        <v>0.01606144078946775</v>
       </c>
     </row>
     <row r="101">
@@ -1879,7 +1879,7 @@
         <v>0.01664911367265891</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>-0.02062269915927131</v>
+        <v>-0.02710332189100653</v>
       </c>
     </row>
     <row r="102">
@@ -1887,10 +1887,10 @@
         <v>44652</v>
       </c>
       <c r="F102" t="n">
-        <v>-0.06831217236867652</v>
+        <v>-0.06831217236867655</v>
       </c>
       <c r="G102" s="2" t="n">
-        <v>-0.03653211832684621</v>
+        <v>-0.02646292599983662</v>
       </c>
     </row>
     <row r="103">
@@ -1901,7 +1901,7 @@
         <v>0.008690514569214445</v>
       </c>
       <c r="G103" s="2" t="n">
-        <v>0.01570605645146273</v>
+        <v>0.02282164628702423</v>
       </c>
     </row>
     <row r="104">
@@ -1909,10 +1909,10 @@
         <v>44713</v>
       </c>
       <c r="F104" t="n">
-        <v>-0.07137486817386951</v>
+        <v>-0.07137486817386952</v>
       </c>
       <c r="G104" s="2" t="n">
-        <v>-0.0409215650664142</v>
+        <v>-0.06828476339409306</v>
       </c>
     </row>
     <row r="105">
@@ -1920,10 +1920,10 @@
         <v>44743</v>
       </c>
       <c r="F105" t="n">
-        <v>0.04215114084727578</v>
+        <v>0.04215114084727579</v>
       </c>
       <c r="G105" s="2" t="n">
-        <v>0.02662232085578096</v>
+        <v>0.02940426991782981</v>
       </c>
     </row>
     <row r="106">
@@ -1934,7 +1934,7 @@
         <v>-0.02062739908050899</v>
       </c>
       <c r="G106" s="2" t="n">
-        <v>-0.01573585020258284</v>
+        <v>-0.02413585137641249</v>
       </c>
     </row>
     <row r="107">
@@ -1945,7 +1945,7 @@
         <v>-0.1006463825719439</v>
       </c>
       <c r="G107" s="2" t="n">
-        <v>-0.07126442838689748</v>
+        <v>-0.06485415306858278</v>
       </c>
     </row>
     <row r="108">
@@ -1956,7 +1956,7 @@
         <v>0.01365951208600223</v>
       </c>
       <c r="G108" s="2" t="n">
-        <v>-0.02370497349991343</v>
+        <v>-0.0267357936899421</v>
       </c>
     </row>
     <row r="109">
@@ -1967,7 +1967,7 @@
         <v>0.1089904939655742</v>
       </c>
       <c r="G109" s="2" t="n">
-        <v>0.1033084224012594</v>
+        <v>0.09325845096025892</v>
       </c>
     </row>
     <row r="110">
@@ -1975,10 +1975,10 @@
         <v>44896</v>
       </c>
       <c r="F110" t="n">
-        <v>0.001797707029514407</v>
+        <v>0.001797707029514409</v>
       </c>
       <c r="G110" s="2" t="n">
-        <v>-0.008270467427200775</v>
+        <v>0.0260866976787971</v>
       </c>
     </row>
     <row r="111">
@@ -1989,7 +1989,7 @@
         <v>0.06470321798872859</v>
       </c>
       <c r="G111" s="2" t="n">
-        <v>0.03575590480213588</v>
+        <v>0.03635769922602901</v>
       </c>
     </row>
     <row r="112">
@@ -2000,7 +2000,7 @@
         <v>-0.04510569340905411</v>
       </c>
       <c r="G112" s="2" t="n">
-        <v>-0.03731852460760221</v>
+        <v>-0.04194365323483813</v>
       </c>
     </row>
     <row r="113">
@@ -2011,7 +2011,7 @@
         <v>0.02698098379847662</v>
       </c>
       <c r="G113" s="2" t="n">
-        <v>0.03506806033475651</v>
+        <v>0.04610412260550841</v>
       </c>
     </row>
     <row r="114">
@@ -2019,10 +2019,10 @@
         <v>45017</v>
       </c>
       <c r="F114" t="n">
-        <v>0.006926623632841845</v>
+        <v>0.006926623632841846</v>
       </c>
       <c r="G114" s="2" t="n">
-        <v>0.02363475003853821</v>
+        <v>0.03620010618689901</v>
       </c>
     </row>
     <row r="115">
@@ -2030,10 +2030,10 @@
         <v>45047</v>
       </c>
       <c r="F115" t="n">
-        <v>-0.008967590973690452</v>
+        <v>-0.00896759097369045</v>
       </c>
       <c r="G115" s="2" t="n">
-        <v>-0.008271366943441895</v>
+        <v>-0.01181653153630413</v>
       </c>
     </row>
     <row r="116">
@@ -2044,7 +2044,7 @@
         <v>0.04594594762545304</v>
       </c>
       <c r="G116" s="2" t="n">
-        <v>0.02284520165073884</v>
+        <v>0.03087450801644917</v>
       </c>
     </row>
     <row r="117">
@@ -2055,7 +2055,7 @@
         <v>0.03775404095517169</v>
       </c>
       <c r="G117" s="2" t="n">
-        <v>0.02904423267542939</v>
+        <v>0.03395158210424336</v>
       </c>
     </row>
     <row r="118">
@@ -2066,7 +2066,7 @@
         <v>-0.03151863659945757</v>
       </c>
       <c r="G118" s="2" t="n">
-        <v>-0.0080735049503928</v>
+        <v>0.008257639532860165</v>
       </c>
     </row>
     <row r="119">
@@ -2077,7 +2077,7 @@
         <v>-0.0172917743383237</v>
       </c>
       <c r="G119" s="2" t="n">
-        <v>-0.01597027054338626</v>
+        <v>-0.006326741811929027</v>
       </c>
     </row>
     <row r="120">
@@ -2088,7 +2088,7 @@
         <v>-0.05045691850664139</v>
       </c>
       <c r="G120" s="2" t="n">
-        <v>-0.02345860679142632</v>
+        <v>-0.01759585980068924</v>
       </c>
     </row>
     <row r="121">
@@ -2096,10 +2096,10 @@
         <v>45231</v>
       </c>
       <c r="F121" t="n">
-        <v>0.06964735184969614</v>
+        <v>0.06964735184969616</v>
       </c>
       <c r="G121" s="2" t="n">
-        <v>-0.00499835983894412</v>
+        <v>-0.09470271811091882</v>
       </c>
     </row>
     <row r="122">
@@ -2107,10 +2107,10 @@
         <v>45261</v>
       </c>
       <c r="F122" t="n">
-        <v>0.05164800673823711</v>
+        <v>0.0516480067382371</v>
       </c>
       <c r="G122" s="2" t="n">
-        <v>0.0567587192559616</v>
+        <v>0.06360078146230626</v>
       </c>
     </row>
     <row r="123">
@@ -2121,7 +2121,7 @@
         <v>0.02182857618970565</v>
       </c>
       <c r="G123" s="2" t="n">
-        <v>0.0111518059730275</v>
+        <v>0.01268294470809439</v>
       </c>
     </row>
     <row r="124">
@@ -2129,10 +2129,10 @@
         <v>45323</v>
       </c>
       <c r="F124" t="n">
-        <v>0.02723204524390988</v>
+        <v>0.02723204524390989</v>
       </c>
       <c r="G124" s="2" t="n">
-        <v>-0.00173655103975348</v>
+        <v>0.004019965729943595</v>
       </c>
     </row>
     <row r="125">
@@ -2143,7 +2143,7 @@
         <v>0.02524587861875428</v>
       </c>
       <c r="G125" s="2" t="n">
-        <v>0.02805259883784097</v>
+        <v>0.04343719854896935</v>
       </c>
     </row>
     <row r="126">
@@ -2154,7 +2154,7 @@
         <v>-0.03475389758867845</v>
       </c>
       <c r="G126" s="2" t="n">
-        <v>-0.02410646856753424</v>
+        <v>-0.03517274115658697</v>
       </c>
     </row>
     <row r="127">
@@ -2165,7 +2165,7 @@
         <v>0.01196510662235034</v>
       </c>
       <c r="G127" s="2" t="n">
-        <v>-0.01423044483292312</v>
+        <v>-0.009961463198129994</v>
       </c>
     </row>
     <row r="128">
@@ -2173,10 +2173,10 @@
         <v>45444</v>
       </c>
       <c r="F128" t="n">
-        <v>-0.005777866332475412</v>
+        <v>-0.005777866332475414</v>
       </c>
       <c r="G128" s="2" t="n">
-        <v>-0.0241460718255382</v>
+        <v>-0.02350414038054454</v>
       </c>
     </row>
     <row r="129">
@@ -2187,7 +2187,7 @@
         <v>0.04816725487792622</v>
       </c>
       <c r="G129" s="2" t="n">
-        <v>0.04899698786181501</v>
+        <v>0.04571925160871092</v>
       </c>
     </row>
     <row r="130">
@@ -2195,10 +2195,10 @@
         <v>45505</v>
       </c>
       <c r="F130" t="n">
-        <v>0.01417762556353758</v>
+        <v>0.01417762556353757</v>
       </c>
       <c r="G130" s="2" t="n">
-        <v>0.01712719537325144</v>
+        <v>0.02468090754113122</v>
       </c>
     </row>
     <row r="131">
@@ -2209,7 +2209,7 @@
         <v>0.02043168751973485</v>
       </c>
       <c r="G131" s="2" t="n">
-        <v>0.01441072319064343</v>
+        <v>0.002513667797089462</v>
       </c>
     </row>
     <row r="132">
@@ -2220,7 +2220,7 @@
         <v>-0.04388213536566083</v>
       </c>
       <c r="G132" s="2" t="n">
-        <v>-0.04314579080071766</v>
+        <v>-0.04028489913569518</v>
       </c>
     </row>
     <row r="133">
@@ -2231,7 +2231,7 @@
         <v>0.003179359263831083</v>
       </c>
       <c r="G133" s="2" t="n">
-        <v>0.01880611660121303</v>
+        <v>0.026351236886701</v>
       </c>
     </row>
     <row r="134">
@@ -2239,10 +2239,10 @@
         <v>45627</v>
       </c>
       <c r="F134" t="n">
-        <v>-0.009904936314324887</v>
+        <v>-0.009904936314324885</v>
       </c>
       <c r="G134" s="2" t="n">
-        <v>-0.01380257567843542</v>
+        <v>-0.01882596239418768</v>
       </c>
     </row>
     <row r="135">
@@ -2253,7 +2253,7 @@
         <v>0.01473281081694431</v>
       </c>
       <c r="G135" s="2" t="n">
-        <v>0.01042421168796662</v>
+        <v>0.04771153523738946</v>
       </c>
     </row>
     <row r="136">
@@ -2261,10 +2261,10 @@
         <v>45689</v>
       </c>
       <c r="F136" t="n">
-        <v>-0.008825849403990397</v>
+        <v>-0.008825849403990395</v>
       </c>
       <c r="G136" s="2" t="n">
-        <v>0.01310553285336153</v>
+        <v>0.04550110652516128</v>
       </c>
     </row>
     <row r="137">
@@ -2275,7 +2275,7 @@
         <v>0.004034043447141258</v>
       </c>
       <c r="G137" s="2" t="n">
-        <v>0.02877367932037785</v>
+        <v>0.04175226815118717</v>
       </c>
     </row>
     <row r="138">
@@ -2283,10 +2283,10 @@
         <v>45748</v>
       </c>
       <c r="F138" t="n">
-        <v>0.05506506557113954</v>
+        <v>0.05506506557113956</v>
       </c>
       <c r="G138" s="2" t="n">
-        <v>0.06032597440740353</v>
+        <v>0.09892414747185098</v>
       </c>
     </row>
     <row r="139">
@@ -2297,7 +2297,7 @@
         <v>0.03866117694017075</v>
       </c>
       <c r="G139" s="2" t="n">
-        <v>0.02099747500810106</v>
+        <v>0.01103063576662626</v>
       </c>
     </row>
     <row r="140">
@@ -2308,7 +2308,7 @@
         <v>0.02285892640434826</v>
       </c>
       <c r="G140" s="2" t="n">
-        <v>0.02969433149487082</v>
+        <v>0.04674698419999613</v>
       </c>
     </row>
     <row r="141">
@@ -2316,10 +2316,10 @@
         <v>45839</v>
       </c>
       <c r="F141" t="n">
-        <v>-0.0002265904128584473</v>
+        <v>-0.0002265904128584478</v>
       </c>
       <c r="G141" s="2" t="n">
-        <v>0.01592855190449243</v>
+        <v>0.01731444447596344</v>
       </c>
     </row>
     <row r="142">
@@ -2327,10 +2327,10 @@
         <v>45870</v>
       </c>
       <c r="F142" t="n">
-        <v>0.0616629502549649</v>
+        <v>0.06166295025496488</v>
       </c>
       <c r="G142" s="2" t="n">
-        <v>0.06241016406866283</v>
+        <v>0.01520985439551823</v>
       </c>
     </row>
     <row r="143">
@@ -2338,10 +2338,10 @@
         <v>45901</v>
       </c>
       <c r="F143" t="n">
-        <v>0.02037228912621098</v>
+        <v>0.02037228912621099</v>
       </c>
       <c r="G143" s="2" t="n">
-        <v>0.01155991273318836</v>
+        <v>0.02317666960089507</v>
       </c>
     </row>
     <row r="144">
@@ -2349,10 +2349,10 @@
         <v>45931</v>
       </c>
       <c r="F144" t="n">
-        <v>0.02807268951678298</v>
+        <v>0.02807268951678299</v>
       </c>
       <c r="G144" s="2" t="n">
-        <v>-0.005064219238300935</v>
+        <v>-0.01314823127804558</v>
       </c>
     </row>
     <row r="145">
@@ -2360,10 +2360,10 @@
         <v>45962</v>
       </c>
       <c r="F145" t="n">
-        <v>-0.006469133677908642</v>
+        <v>-0.006469133677908643</v>
       </c>
       <c r="G145" s="2" t="n">
-        <v>0.02685021106538299</v>
+        <v>0.02688328647259337</v>
       </c>
     </row>
     <row r="146">
@@ -2371,10 +2371,10 @@
         <v>45992</v>
       </c>
       <c r="F146" s="4" t="n">
-        <v>0.007292430941722384</v>
+        <v>0.007292430941722383</v>
       </c>
       <c r="G146" s="5" t="n">
-        <v>-0.007060512442369751</v>
+        <v>0.0133575088389439</v>
       </c>
     </row>
   </sheetData>

</xml_diff>